<commit_message>
Rules schema overhaul, Claude auto-suggest, address column
- Replace per-rule empresa with descricao field; descricao matches now
  take priority over palavra_chave matches.
- When the description cell actually holds an address (matches the
  mapped Endereco column or address regex), skip descricao rules and
  fall through directly to palavra_chave.
- Add Endereco (opcional) column dropdown in Section 2; auto-detect via
  new regex hints in extract_fixed_expenses.COLUMN_HINTS; carry through
  to preview and Excel export.
- New tools/categorize_with_claude.py wraps the Anthropic SDK to
  suggest categories for unmatched rows in batches; opt-in checkbox in
  Section 4 (requires ANTHROPIC_API_KEY in .env or Streamlit secrets).
- Regenerate config/categorias.xlsx with the new 3-column schema.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/categorias.xlsx
+++ b/config/categorias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,14 +429,14 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>empresa</t>
+          <t>descricao</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>maria</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -444,79 +444,46 @@
           <t>Aluguel</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>bruno ABC</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Rafael</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Seguros</t>
+          <t>Energia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bruno ABC</t>
+          <t>energia eletrica</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Lucas</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Folha de Pagamento</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bruno ABC</t>
+          <t>vivo fibra</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Maria</t>
+          <t>condom</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Agua</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Thais abc</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Beatriz</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Luz</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Thais abc</t>
-        </is>
-      </c>
+          <t>Condomínio</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Seed categorias.xlsx with 28 starter rules
Pre-populates the sidebar with the user's standard expense categories
(Aluguel, IPTU, Enel, Sabesp, Claro/Net, Vivo, Hagana, Grupo Gabriel,
Sanear, Supricorp/Gimba, Seguro Incêndio, etc.) so the user doesn't
have to type them on first use.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/categorias.xlsx
+++ b/config/categorias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,56 +434,408 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>maria</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Aluguel</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>aluguel</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Energia</t>
+          <t>IPTU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>energia eletrica</t>
+          <t>iptu</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>enel</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Enel</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>vivo fibra</t>
+          <t>enel</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>condom</t>
+          <t>sabesp</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Condomínio</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>Sabesp</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sabesp</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Claro/Net</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>claro</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">net </t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Claro/Net</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>net</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Telefone</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>telefone</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hagana</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hagana</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>hagana</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Limpa vidros</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>limpa vidros</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Segurança</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>seguranca</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>gabriel</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Grupo Gabriel</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>grupo gabriel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sanear</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sanear (diversos qdo precisa)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>sanear</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>supricorp</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Supricorp/Gimba</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>supricorp</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>gimba</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Supricorp/Gimba</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>gimba</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pão de queijo para clientes</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>pao de queijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Água personalizada para cliente</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>agua personalizada</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Locação de impressora+cartucho</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>impressora</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Locação de impressora+cartucho</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>cartucho</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Seguro Incêndio</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>seguro incendio</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Auto de licença de funcionamento</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>licenca de funcionamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Troca Extintores</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>extintor</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Laudo bombeiro</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>laudo bombeiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Galão de água</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>galao</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Galão de água</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>galão</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Garagens carros Taag</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>garagem</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cowork</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>cowork</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Depósito</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>deposito</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>